<commit_message>
feat: Phase 3 — Zernike PSF, field-dependent WFE, chromatic aberrations, folded MTF, access geometry
Phase 3A: Optics element model (ElementTransferMode, NearfieldResult per-element),
defocus module, Zernike polynomial evaluation (Noll-indexed), polychromatic PSF
with per-wavelength storage (PolychromaticPSFResult dataclass).

Phase 3B: GSD cross/along-track with Earth curvature, ground range, swath width,
access rate calculators. PlatformStage jitter + smear wiring. Atmosphere/detector
schema extensions (path_zenith_rad, IPC kernel size).

Phase 3C: Field-dependent WFE (at_field/at_field_nearest lookup), chromatic
Zernikes for refractive systems (ElementTransferMode.REFRACTIVE), aliased/folded
MTF (compute_folded_mtf with alias fraction), IO element config loader.

Closes gaps: 14 (folded MTF), 16 (per-wavelength PSF), 24 (Zernike-to-PSF),
25 (field-dependent WFE). Scenarios 1.4, 3.4, 5.1, 5.2, 7.3 updated.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scenarios/03_raj_mission_planner/3.4_off_nadir_agility/outputs/off_nadir_results.xlsx
+++ b/scenarios/03_raj_mission_planner/3.4_off_nadir_agility/outputs/off_nadir_results.xlsx
@@ -608,7 +608,7 @@
         <v>5.86</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>5.87</v>
+        <v>5.86</v>
       </c>
       <c r="N3" s="2" t="n">
         <v>15374</v>
@@ -649,10 +649,10 @@
         <v>0.6457000000000001</v>
       </c>
       <c r="L4" s="2" t="n">
+        <v>5.84</v>
+      </c>
+      <c r="M4" s="2" t="n">
         <v>5.85</v>
-      </c>
-      <c r="M4" s="2" t="n">
-        <v>5.89</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>16005</v>
@@ -693,10 +693,10 @@
         <v>0.6457000000000001</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>5.82</v>
+        <v>5.79</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>5.9</v>
+        <v>5.81</v>
       </c>
       <c r="N5" s="2" t="n">
         <v>16623</v>
@@ -737,10 +737,10 @@
         <v>0.6457000000000001</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>5.78</v>
+        <v>5.72</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>5.91</v>
+        <v>5.76</v>
       </c>
       <c r="N6" s="2" t="n">
         <v>17219</v>
@@ -781,10 +781,10 @@
         <v>0.6457000000000001</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>5.71</v>
+        <v>5.62</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>5.92</v>
+        <v>5.68</v>
       </c>
       <c r="N7" s="2" t="n">
         <v>17789</v>
@@ -825,10 +825,10 @@
         <v>0.6457000000000001</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>5.62</v>
+        <v>5.49</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>5.93</v>
+        <v>5.57</v>
       </c>
       <c r="N8" s="2" t="n">
         <v>18329</v>
@@ -869,10 +869,10 @@
         <v>0.6457000000000001</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>5.5</v>
+        <v>5.32</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>5.94</v>
+        <v>5.44</v>
       </c>
       <c r="N9" s="2" t="n">
         <v>18837</v>
@@ -913,10 +913,10 @@
         <v>0.6457000000000001</v>
       </c>
       <c r="L10" s="2" t="n">
-        <v>5.36</v>
+        <v>5.12</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>5.95</v>
+        <v>5.27</v>
       </c>
       <c r="N10" s="2" t="n">
         <v>19311</v>
@@ -957,10 +957,10 @@
         <v>0.6457000000000001</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>5.19</v>
+        <v>4.86</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>5.96</v>
+        <v>5.06</v>
       </c>
       <c r="N11" s="2" t="n">
         <v>19754</v>

</xml_diff>